<commit_message>
improvements to Frame Broadcaster, minor changes on tutorials
</commit_message>
<xml_diff>
--- a/robotics/from_code_to_robot_robotics_schedule.xlsx
+++ b/robotics/from_code_to_robot_robotics_schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Const\Desktop\Work\GitIoc\from-code-to-robot\robotics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Const\Desktop\Work\GitIoc\robotics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A992B0E-5709-422E-94A6-FBA4FC58121A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B28D50C-DCED-4D51-9005-EDEA8412D112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="schedule" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="132">
   <si>
     <t>Set-up</t>
   </si>
@@ -218,12 +218,6 @@
     <t>Gazebo</t>
   </si>
   <si>
-    <t>Programming</t>
-  </si>
-  <si>
-    <t>URSim / Real</t>
-  </si>
-  <si>
     <t>3. DIFFERENTIAL KINEMATICS</t>
   </si>
   <si>
@@ -423,6 +417,30 @@
   </si>
   <si>
     <t xml:space="preserve">give picture of UR model and let them set up the robot themselves </t>
+  </si>
+  <si>
+    <t>Planar arm + Antro&amp;Wrist</t>
+  </si>
+  <si>
+    <t>Define the reachable Workspace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">make function to segment the path into intermediate steps </t>
+  </si>
+  <si>
+    <t>make a function to compute the joint angles for these steps</t>
+  </si>
+  <si>
+    <t>give trajectory in jointspace</t>
+  </si>
+  <si>
+    <t>Rviz with teleop twist keyboard or turtlesim</t>
+  </si>
+  <si>
+    <t>track joint velocities while doing a rectengular motion (through singularity) --&gt; part of tutorial</t>
+  </si>
+  <si>
+    <t>Setup Jacobians, Determinant of Jacobian at different points, get cartesian position for constant velocity, Rank of Jacobian, Check the Velocity --&gt; compute trajectory in an axis and monitor the velocities</t>
   </si>
 </sst>
 </file>
@@ -532,7 +550,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -565,6 +583,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1162,22 +1183,22 @@
     <row r="28" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1221,12 +1242,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.88671875" customWidth="1"/>
     <col min="2" max="2" width="59.88671875" customWidth="1"/>
     <col min="3" max="3" width="27.5546875" customWidth="1"/>
+    <col min="4" max="4" width="57.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1314,62 +1336,73 @@
       </c>
     </row>
     <row r="16" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:3" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>53</v>
       </c>
       <c r="C24" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D24" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>55</v>
       </c>
       <c r="C25" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D25" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>52</v>
       </c>
       <c r="C26" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>57</v>
-      </c>
-      <c r="C27" t="s">
-        <v>58</v>
+      <c r="D26" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D27" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D28" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -1399,17 +1432,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.44140625" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="16.88671875" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1422,12 +1456,12 @@
         <v>14</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1439,66 +1473,75 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>72</v>
+        <v>70</v>
+      </c>
+      <c r="D20" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -1525,7 +1568,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1543,7 +1586,7 @@
     </row>
     <row r="4" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>17</v>
@@ -1551,12 +1594,12 @@
     </row>
     <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1596,7 +1639,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1614,7 +1657,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>17</v>
@@ -1622,12 +1665,12 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1667,13 +1710,13 @@
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C1" s="18" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D1" s="18"/>
       <c r="E1" s="18"/>
       <c r="F1" s="18"/>
       <c r="G1" s="18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H1" s="18"/>
       <c r="I1" s="18"/>
@@ -1682,53 +1725,53 @@
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C2" s="18" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D2" s="18"/>
       <c r="E2" s="18" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F2" s="18"/>
       <c r="G2" s="18" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H2" s="18"/>
       <c r="I2" s="18" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J2" s="18"/>
       <c r="K2" s="8"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C3" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K3" s="8"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C4" s="10">
         <v>1</v>
@@ -1750,7 +1793,7 @@
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1764,7 +1807,7 @@
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -1778,7 +1821,7 @@
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C7" s="10">
         <v>6</v>
@@ -1808,7 +1851,7 @@
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="11" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -1822,7 +1865,7 @@
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1836,7 +1879,7 @@
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1850,7 +1893,7 @@
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" s="11" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1864,7 +1907,7 @@
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1878,7 +1921,7 @@
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" s="11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -1892,7 +1935,7 @@
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -1906,7 +1949,7 @@
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" s="11" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -1920,7 +1963,7 @@
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16" s="11" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -1934,7 +1977,7 @@
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -1948,7 +1991,7 @@
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" s="11" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1962,7 +2005,7 @@
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B19" s="11" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -1976,7 +2019,7 @@
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" s="11" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -1990,7 +2033,7 @@
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B21" s="11" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -2004,7 +2047,7 @@
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C22" s="10">
         <v>3</v>
@@ -2026,7 +2069,7 @@
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="11" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -2040,7 +2083,7 @@
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B24" s="11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -2054,7 +2097,7 @@
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -2068,7 +2111,7 @@
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B26" s="11" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
@@ -2082,7 +2125,7 @@
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" s="11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -2096,7 +2139,7 @@
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B28" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C28" s="10">
         <v>4</v>
@@ -2126,7 +2169,7 @@
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -2140,7 +2183,7 @@
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B30" s="11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -2154,7 +2197,7 @@
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -2168,7 +2211,7 @@
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B32" s="11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -2182,7 +2225,7 @@
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -2196,7 +2239,7 @@
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" s="11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -2210,7 +2253,7 @@
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" s="11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -2224,7 +2267,7 @@
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -2238,7 +2281,7 @@
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" s="11" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -2252,7 +2295,7 @@
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" s="12" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C38" s="13">
         <f>C4+C7+C22+C28</f>
@@ -2278,7 +2321,7 @@
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C39" s="15"/>
       <c r="D39" s="15">
@@ -2333,6 +2376,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002DE95F3A66967442A10BA11B8E4FFC36" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5c2e22b68f6e8758347731c1e29ce2f5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c4e57b37-1674-4273-ab2d-7b2370a90a1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="97258493908a7724e3cfd4a364c35939" ns2:_="">
     <xsd:import namespace="c4e57b37-1674-4273-ab2d-7b2370a90a1c"/>
@@ -2470,12 +2519,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F698B387-0CAC-476E-903C-4D869C8807D2}">
   <ds:schemaRefs>
@@ -2485,6 +2528,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C29AC991-11A8-4EE5-92EB-DD6DA06A5013}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51128220-6E17-45B1-950E-336F1B236F1D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2500,13 +2552,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C29AC991-11A8-4EE5-92EB-DD6DA06A5013}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added solutions for kinematics exercises 1, added function for checking exercises getIndex for complex inputs and function calls
</commit_message>
<xml_diff>
--- a/robotics/from_code_to_robot_robotics_schedule.xlsx
+++ b/robotics/from_code_to_robot_robotics_schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Const\Desktop\Work\GitIoc\robotics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B28D50C-DCED-4D51-9005-EDEA8412D112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{249CCA66-89E3-40E1-94E3-0435596F0F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="schedule" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="137">
   <si>
     <t>Set-up</t>
   </si>
@@ -441,6 +441,21 @@
   </si>
   <si>
     <t>Setup Jacobians, Determinant of Jacobian at different points, get cartesian position for constant velocity, Rank of Jacobian, Check the Velocity --&gt; compute trajectory in an axis and monitor the velocities</t>
+  </si>
+  <si>
+    <t>functions for coriolis, friction, gravity, innertia</t>
+  </si>
+  <si>
+    <t>IK algorithm pseudoinverse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">balance a mass gravity on gazebo at different configurations </t>
+  </si>
+  <si>
+    <t>parameterization example two_link_manipulator.m</t>
+  </si>
+  <si>
+    <t>find the acceleration to track a trajectory</t>
   </si>
 </sst>
 </file>
@@ -581,11 +596,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -971,13 +986,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="20.88671875" customWidth="1"/>
+    <col min="1" max="1" width="4.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -985,7 +1000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>2</v>
       </c>
@@ -993,7 +1008,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>4</v>
       </c>
@@ -1001,7 +1016,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>6</v>
       </c>
@@ -1009,7 +1024,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>8</v>
       </c>
@@ -1017,7 +1032,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>10</v>
       </c>
@@ -1038,24 +1053,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.109375" customWidth="1"/>
-    <col min="2" max="2" width="58.44140625" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="2" max="2" width="58.42578125" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1063,7 +1078,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1071,37 +1086,37 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B7" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1109,17 +1124,17 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1127,43 +1142,43 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>36</v>
       </c>
@@ -1171,7 +1186,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>38</v>
       </c>
@@ -1179,43 +1194,43 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="33" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="36" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="37" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="49" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="50" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
@@ -1243,25 +1258,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.88671875" customWidth="1"/>
-    <col min="2" max="2" width="59.88671875" customWidth="1"/>
-    <col min="3" max="3" width="27.5546875" customWidth="1"/>
-    <col min="4" max="4" width="57.33203125" customWidth="1"/>
+    <col min="1" max="1" width="21.85546875" customWidth="1"/>
+    <col min="2" max="2" width="59.85546875" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" customWidth="1"/>
+    <col min="4" max="4" width="57.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1269,12 +1284,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1282,32 +1297,32 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1315,54 +1330,54 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:4" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="17" spans="1:4" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>53</v>
       </c>
@@ -1373,7 +1388,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>55</v>
       </c>
@@ -1384,7 +1399,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>52</v>
       </c>
@@ -1395,12 +1410,12 @@
         <v>126</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D27" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D28" t="s">
         <v>128</v>
       </c>
@@ -1432,26 +1447,26 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1459,70 +1474,70 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>67</v>
       </c>
       <c r="C18" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="18" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>63</v>
       </c>
@@ -1533,7 +1548,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>69</v>
       </c>
@@ -1542,6 +1557,11 @@
       </c>
       <c r="D20" t="s">
         <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D21" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1559,24 +1579,24 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.109375" customWidth="1"/>
-    <col min="2" max="2" width="56.6640625" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="56.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1584,7 +1604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -1592,24 +1612,44 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="6" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" s="6" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1631,23 +1671,23 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.109375" customWidth="1"/>
-    <col min="2" max="2" width="34.109375" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1655,7 +1695,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -1663,22 +1703,22 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B5" s="6" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" s="6" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" s="5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>33</v>
       </c>
@@ -1702,47 +1742,47 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B1:K39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" customWidth="1"/>
-    <col min="2" max="2" width="34.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="34.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="C1" s="18" t="s">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="C1" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18" t="s">
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
       <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="C2" s="18" t="s">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="C2" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18" t="s">
+      <c r="D2" s="19"/>
+      <c r="E2" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18" t="s">
+      <c r="F2" s="19"/>
+      <c r="G2" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18" t="s">
+      <c r="H2" s="19"/>
+      <c r="I2" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="J2" s="18"/>
+      <c r="J2" s="19"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>82</v>
       </c>
@@ -1769,7 +1809,7 @@
       </c>
       <c r="K3" s="8"/>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B4" s="9" t="s">
         <v>84</v>
       </c>
@@ -1791,7 +1831,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="8"/>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B5" s="11" t="s">
         <v>85</v>
       </c>
@@ -1805,7 +1845,7 @@
       <c r="J5" s="1"/>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
         <v>86</v>
       </c>
@@ -1819,7 +1859,7 @@
       <c r="J6" s="1"/>
       <c r="K6" s="8"/>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B7" s="9" t="s">
         <v>87</v>
       </c>
@@ -1849,7 +1889,7 @@
       </c>
       <c r="K7" s="8"/>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B8" s="11" t="s">
         <v>88</v>
       </c>
@@ -1863,7 +1903,7 @@
       <c r="J8" s="1"/>
       <c r="K8" s="8"/>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B9" s="11" t="s">
         <v>89</v>
       </c>
@@ -1877,7 +1917,7 @@
       <c r="J9" s="1"/>
       <c r="K9" s="8"/>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B10" s="11" t="s">
         <v>90</v>
       </c>
@@ -1891,7 +1931,7 @@
       <c r="J10" s="1"/>
       <c r="K10" s="8"/>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B11" s="11" t="s">
         <v>91</v>
       </c>
@@ -1905,7 +1945,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="8"/>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B12" s="11" t="s">
         <v>92</v>
       </c>
@@ -1919,7 +1959,7 @@
       <c r="J12" s="1"/>
       <c r="K12" s="8"/>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B13" s="11" t="s">
         <v>93</v>
       </c>
@@ -1933,7 +1973,7 @@
       <c r="J13" s="1"/>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
         <v>94</v>
       </c>
@@ -1947,7 +1987,7 @@
       <c r="J14" s="1"/>
       <c r="K14" s="8"/>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B15" s="11" t="s">
         <v>95</v>
       </c>
@@ -1961,7 +2001,7 @@
       <c r="J15" s="1"/>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
         <v>96</v>
       </c>
@@ -1975,7 +2015,7 @@
       <c r="J16" s="1"/>
       <c r="K16" s="8"/>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B17" s="11" t="s">
         <v>97</v>
       </c>
@@ -1989,7 +2029,7 @@
       <c r="J17" s="1"/>
       <c r="K17" s="8"/>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B18" s="11" t="s">
         <v>98</v>
       </c>
@@ -2003,7 +2043,7 @@
       <c r="J18" s="1"/>
       <c r="K18" s="8"/>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B19" s="11" t="s">
         <v>99</v>
       </c>
@@ -2017,7 +2057,7 @@
       <c r="J19" s="1"/>
       <c r="K19" s="8"/>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B20" s="11" t="s">
         <v>100</v>
       </c>
@@ -2031,7 +2071,7 @@
       <c r="J20" s="1"/>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
         <v>101</v>
       </c>
@@ -2045,7 +2085,7 @@
       <c r="J21" s="1"/>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B22" s="9" t="s">
         <v>102</v>
       </c>
@@ -2067,7 +2107,7 @@
       <c r="J22" s="10"/>
       <c r="K22" s="8"/>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B23" s="11" t="s">
         <v>103</v>
       </c>
@@ -2081,7 +2121,7 @@
       <c r="J23" s="1"/>
       <c r="K23" s="8"/>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
         <v>104</v>
       </c>
@@ -2095,7 +2135,7 @@
       <c r="J24" s="1"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B25" s="11" t="s">
         <v>105</v>
       </c>
@@ -2109,7 +2149,7 @@
       <c r="J25" s="1"/>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
         <v>106</v>
       </c>
@@ -2123,7 +2163,7 @@
       <c r="J26" s="1"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
         <v>107</v>
       </c>
@@ -2137,7 +2177,7 @@
       <c r="J27" s="1"/>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B28" s="9" t="s">
         <v>108</v>
       </c>
@@ -2167,7 +2207,7 @@
       </c>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B29" s="11" t="s">
         <v>109</v>
       </c>
@@ -2181,7 +2221,7 @@
       <c r="J29" s="1"/>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B30" s="11" t="s">
         <v>110</v>
       </c>
@@ -2195,7 +2235,7 @@
       <c r="J30" s="1"/>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B31" s="11" t="s">
         <v>111</v>
       </c>
@@ -2209,7 +2249,7 @@
       <c r="J31" s="1"/>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B32" s="11" t="s">
         <v>112</v>
       </c>
@@ -2223,7 +2263,7 @@
       <c r="J32" s="1"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B33" s="11" t="s">
         <v>113</v>
       </c>
@@ -2237,7 +2277,7 @@
       <c r="J33" s="1"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B34" s="11" t="s">
         <v>114</v>
       </c>
@@ -2251,7 +2291,7 @@
       <c r="J34" s="1"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B35" s="11" t="s">
         <v>115</v>
       </c>
@@ -2265,7 +2305,7 @@
       <c r="J35" s="1"/>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B36" s="11" t="s">
         <v>116</v>
       </c>
@@ -2279,7 +2319,7 @@
       <c r="J36" s="1"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B37" s="11" t="s">
         <v>117</v>
       </c>
@@ -2293,7 +2333,7 @@
       <c r="J37" s="1"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B38" s="12" t="s">
         <v>118</v>
       </c>
@@ -2319,7 +2359,7 @@
       <c r="J38" s="13"/>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B39" s="14" t="s">
         <v>119</v>
       </c>
@@ -2376,12 +2416,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002DE95F3A66967442A10BA11B8E4FFC36" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5c2e22b68f6e8758347731c1e29ce2f5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c4e57b37-1674-4273-ab2d-7b2370a90a1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="97258493908a7724e3cfd4a364c35939" ns2:_="">
     <xsd:import namespace="c4e57b37-1674-4273-ab2d-7b2370a90a1c"/>
@@ -2519,6 +2553,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F698B387-0CAC-476E-903C-4D869C8807D2}">
   <ds:schemaRefs>
@@ -2528,15 +2568,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C29AC991-11A8-4EE5-92EB-DD6DA06A5013}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51128220-6E17-45B1-950E-336F1B236F1D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2552,4 +2583,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C29AC991-11A8-4EE5-92EB-DD6DA06A5013}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
started Jacobians Tutorials including images. minor changes to previous exercises (Trajectory Planning)
</commit_message>
<xml_diff>
--- a/robotics/from_code_to_robot_robotics_schedule.xlsx
+++ b/robotics/from_code_to_robot_robotics_schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Const\Desktop\Work\GitIoc\robotics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{249CCA66-89E3-40E1-94E3-0435596F0F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A37097F-30B8-4FF3-8845-DA2519C65697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" tabRatio="500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="schedule" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="147">
   <si>
     <t>Set-up</t>
   </si>
@@ -456,6 +456,36 @@
   </si>
   <si>
     <t>find the acceleration to track a trajectory</t>
+  </si>
+  <si>
+    <t>Dynamic Matrices (coriolis, friction, gravity, innertia)--&gt; lagrange</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parameterization </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dynamic Identification </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Understand when to apply centeralized control </t>
+  </si>
+  <si>
+    <t>(tuning of PID controller, rootlocus)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">centeralized control </t>
+  </si>
+  <si>
+    <t>decentralized control -&gt; couplings are treated as disturbances, feedforward terms for better performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">centeralized control scheme in simulink with gravity compensation PD </t>
+  </si>
+  <si>
+    <t xml:space="preserve">inverse dynamic control </t>
+  </si>
+  <si>
+    <t>(dynamic model in operational space)</t>
   </si>
 </sst>
 </file>
@@ -1627,6 +1657,21 @@
         <v>29</v>
       </c>
     </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>139</v>
+      </c>
+    </row>
     <row r="18" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>33</v>
@@ -1670,11 +1715,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.140625" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="2" max="2" width="117.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -1718,9 +1763,44 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2416,6 +2496,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002DE95F3A66967442A10BA11B8E4FFC36" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5c2e22b68f6e8758347731c1e29ce2f5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c4e57b37-1674-4273-ab2d-7b2370a90a1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="97258493908a7724e3cfd4a364c35939" ns2:_="">
     <xsd:import namespace="c4e57b37-1674-4273-ab2d-7b2370a90a1c"/>
@@ -2553,12 +2639,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F698B387-0CAC-476E-903C-4D869C8807D2}">
   <ds:schemaRefs>
@@ -2568,6 +2648,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C29AC991-11A8-4EE5-92EB-DD6DA06A5013}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51128220-6E17-45B1-950E-336F1B236F1D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2583,13 +2672,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C29AC991-11A8-4EE5-92EB-DD6DA06A5013}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>